<commit_message>
Update merchant success probabilities
</commit_message>
<xml_diff>
--- a/Team2_確率 (1).xlsx
+++ b/Team2_確率 (1).xlsx
@@ -1112,7 +1112,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75107F64-8075-4579-9F36-30D9A5DB9C16}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{75107F64-8075-4579-9F36-30D9A5DB9C16}">
   <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <sheetData>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="C2">
         <f>2/6</f>
-        <v>0.33333333333333331</v>
+        <v>0.1666666667</v>
       </c>
       <c r="D2">
         <f>3</f>
@@ -1186,7 +1186,7 @@
       </c>
       <c r="C4">
         <f>4/6</f>
-        <v>0.66666666666666663</v>
+        <v>0.3333333333</v>
       </c>
       <c r="D4">
         <f>5</f>
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C5">
         <f>2/6</f>
-        <v>0.33333333333333331</v>
+        <v>0.3333333333</v>
       </c>
       <c r="D5">
         <f>3</f>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C6">
         <f>1/2</f>
-        <v>0.5</v>
+        <v>0.6666666667</v>
       </c>
       <c r="D6">
         <f>2</f>
@@ -1253,7 +1253,7 @@
       </c>
       <c r="C7">
         <f>4/6</f>
-        <v>0.66666666666666663</v>
+        <v>0.5</v>
       </c>
       <c r="D7">
         <f>5</f>

</xml_diff>